<commit_message>
Test data: Anna all 3 secondary curriculums; Alexis one secondary
Anna Harbort: Acute Care + Ambulatory + Extended Care (all 3 slices filled)
Alexis Hollie: Ambulatory only (one slice filled)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cert-data/FY26-Healthcare-Certification-Courses_2026-05.xlsx
+++ b/cert-data/FY26-Healthcare-Certification-Courses_2026-05.xlsx
@@ -15,7 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="19">
     <font>
       <name val="Aptos Narrow"/>
@@ -514,7 +516,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -538,6 +540,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1787,14 +1790,20 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="AB5" s="9" t="n">
+        <v>46162</v>
+      </c>
       <c r="AD5" s="3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AE5" s="9" t="n">
+        <v>46174</v>
       </c>
       <c r="AG5" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2038,10 +2047,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AB7" s="7" t="n"/>
+      <c r="AB7" s="7" t="n">
+        <v>46122</v>
+      </c>
       <c r="AD7" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE7" s="7" t="n"/>

</xml_diff>